<commit_message>
Hoàn thành tất cả
Co-authored-by: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/outputs/project_docs_20260423/Tai-lieu-cau-truc-du-an-BTLAND.xlsx
+++ b/outputs/project_docs_20260423/Tai-lieu-cau-truc-du-an-BTLAND.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan" sheetId="1" r:id="Rea1ced06b7a244c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc file" sheetId="2" r:id="Raa348222d05c4d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ghi chu" sheetId="3" r:id="R5bcd10f796024507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan" sheetId="1" r:id="R15e237507fa34a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc file" sheetId="2" r:id="R462c975cf36a4158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ghi chu" sheetId="3" r:id="R9987621f3a6a41ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,7 +430,7 @@
         <x:v>Tổng số file được mô tả</x:v>
       </x:c>
       <x:c r="B5" s="33" t="n">
-        <x:v>82</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C5" s="33"/>
       <x:c r="D5" s="32"/>
@@ -540,7 +540,7 @@
         <x:v>Java/Activity</x:v>
       </x:c>
       <x:c r="B15" s="33" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C15" s="33" t="str">
         <x:v>Số file thuộc nhóm Java/Activity</x:v>
@@ -552,7 +552,7 @@
         <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="B16" s="33" t="n">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C16" s="33" t="str">
         <x:v>Số file thuộc nhóm Java/Adapter</x:v>
@@ -561,49 +561,49 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="33" t="str">
-        <x:v>Java/Fragment</x:v>
+        <x:v>Java/Application</x:v>
       </x:c>
       <x:c r="B17" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="33" t="str">
-        <x:v>Số file thuộc nhóm Java/Fragment</x:v>
+        <x:v>Số file thuộc nhóm Java/Application</x:v>
       </x:c>
       <x:c r="D17" s="32"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="33" t="str">
-        <x:v>Java/Model</x:v>
+        <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="B18" s="33" t="n">
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="33" t="str">
-        <x:v>Số file thuộc nhóm Java/Model</x:v>
+        <x:v>Số file thuộc nhóm Java/Fragment</x:v>
       </x:c>
       <x:c r="D18" s="32"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="33" t="str">
-        <x:v>Java/Utility</x:v>
+        <x:v>Java/Model</x:v>
       </x:c>
       <x:c r="B19" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C19" s="33" t="str">
-        <x:v>Số file thuộc nhóm Java/Utility</x:v>
+        <x:v>Số file thuộc nhóm Java/Model</x:v>
       </x:c>
       <x:c r="D19" s="32"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="33" t="str">
-        <x:v>Khác</x:v>
+        <x:v>Java/Utility</x:v>
       </x:c>
       <x:c r="B20" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C20" s="33" t="str">
-        <x:v>Số file thuộc nhóm Khác</x:v>
+        <x:v>Số file thuộc nhóm Java/Utility</x:v>
       </x:c>
       <x:c r="D20" s="32"/>
     </x:row>
@@ -633,92 +633,98 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="33" t="str">
-        <x:v>Resource/Drawable</x:v>
+        <x:v>Resource/Color</x:v>
       </x:c>
       <x:c r="B23" s="33" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/Drawable</x:v>
+        <x:v>Số file thuộc nhóm Resource/Color</x:v>
       </x:c>
       <x:c r="D23" s="32"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="33" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="B24" s="33" t="n">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C24" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/Layout</x:v>
+        <x:v>Số file thuộc nhóm Resource/Drawable</x:v>
       </x:c>
       <x:c r="D24" s="32"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33" t="str">
-        <x:v>Resource/Menu</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="B25" s="33" t="n">
-        <x:v>1</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C25" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/Menu</x:v>
+        <x:v>Số file thuộc nhóm Resource/Layout</x:v>
       </x:c>
       <x:c r="D25" s="32"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="33" t="str">
-        <x:v>Resource/Theme</x:v>
+        <x:v>Resource/Menu</x:v>
       </x:c>
       <x:c r="B26" s="33" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C26" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/Theme</x:v>
+        <x:v>Số file thuộc nhóm Resource/Menu</x:v>
       </x:c>
       <x:c r="D26" s="32"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="33" t="str">
-        <x:v>Resource/Value</x:v>
+        <x:v>Resource/Theme</x:v>
       </x:c>
       <x:c r="B27" s="33" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C27" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/Value</x:v>
+        <x:v>Số file thuộc nhóm Resource/Theme</x:v>
       </x:c>
       <x:c r="D27" s="32"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="33" t="str">
-        <x:v>Resource/XML</x:v>
+        <x:v>Resource/Value</x:v>
       </x:c>
       <x:c r="B28" s="33" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C28" s="33" t="str">
-        <x:v>Số file thuộc nhóm Resource/XML</x:v>
+        <x:v>Số file thuộc nhóm Resource/Value</x:v>
       </x:c>
       <x:c r="D28" s="32"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="33" t="str">
+        <x:v>Resource/XML</x:v>
+      </x:c>
+      <x:c r="B29" s="33" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C29" s="33" t="str">
+        <x:v>Số file thuộc nhóm Resource/XML</x:v>
+      </x:c>
+      <x:c r="D29" s="32"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="33" t="str">
         <x:v>Tài liệu</x:v>
       </x:c>
-      <x:c r="B29" s="33" t="n">
+      <x:c r="B30" s="33" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C29" s="33" t="str">
+      <x:c r="C30" s="33" t="str">
         <x:v>Số file thuộc nhóm Tài liệu</x:v>
       </x:c>
-      <x:c r="D29" s="32"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="33"/>
-      <x:c r="B30" s="33"/>
-      <x:c r="C30" s="33"/>
       <x:c r="D30" s="32"/>
     </x:row>
   </x:sheetData>
@@ -941,7 +947,7 @@
         <x:v>Message.java, Conversation.java, MessageAdapter.java, firestore.rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="214.84375" hidden="0" customHeight="1">
+    <x:row r="11" ht="201.416015625" hidden="0" customHeight="1">
       <x:c r="A11" s="50" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -955,7 +961,7 @@
         <x:v>Màn hình tạo bài đăng mới.</x:v>
       </x:c>
       <x:c r="E11" s="47" t="str">
-        <x:v>Nhập thông tin bài, chọn/chụp ảnh, lấy GPS, tạo ảnh 360 từ ảnh thường hoặc chọn panorama, rồi upload lên Firebase.</x:v>
+        <x:v>Nhập thông tin bài, chọn/chụp ảnh thường, chọn ảnh 360 từ thư viện, lấy GPS rồi upload toàn bộ lên Firebase.</x:v>
       </x:c>
       <x:c r="F11" s="47" t="str">
         <x:v>activity_create_post.xml, Post.java, FirebaseStorageHelper.java</x:v>
@@ -1061,7 +1067,7 @@
         <x:v>item_post.xml, PostRepository.java, PostAdapter.java</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="120.849609375" hidden="0" customHeight="1">
+    <x:row r="17" ht="134.27734375" hidden="0" customHeight="1">
       <x:c r="A17" s="50" t="n">
         <x:v>16</x:v>
       </x:c>
@@ -1069,19 +1075,19 @@
         <x:v>Java/Activity</x:v>
       </x:c>
       <x:c r="C17" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/activities/PostDetailActivity.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/activities/PanoramaViewActivity.java</x:v>
       </x:c>
       <x:c r="D17" s="47" t="str">
-        <x:v>Màn hình chi tiết bài đăng.</x:v>
+        <x:v>Màn hình xem ảnh panorama/360.</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Xem thông tin đầy đủ, ảnh, panorama và liên hệ chủ bài qua chat.</x:v>
+        <x:v>Hiển thị ảnh 360 theo kiểu cuộn ngang và hỗ trợ gyroscope nếu thiết bị có.</x:v>
       </x:c>
       <x:c r="F17" s="47" t="str">
-        <x:v>activity_post_detail.xml, ChatActivity.java, PanoramaViewActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>activity_panorama_view.xml, PostDetailActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="120.849609375" hidden="0" customHeight="1">
       <x:c r="A18" s="50" t="n">
         <x:v>17</x:v>
       </x:c>
@@ -1089,16 +1095,16 @@
         <x:v>Java/Activity</x:v>
       </x:c>
       <x:c r="C18" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/activities/RegisterActivity.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/activities/PostDetailActivity.java</x:v>
       </x:c>
       <x:c r="D18" s="47" t="str">
-        <x:v>Màn hình đăng ký tài khoản mới.</x:v>
+        <x:v>Màn hình chi tiết bài đăng.</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Tạo user Firebase Auth và hồ sơ user trên Firestore.</x:v>
+        <x:v>Xem thông tin đầy đủ, ảnh, panorama và liên hệ chủ bài qua chat.</x:v>
       </x:c>
       <x:c r="F18" s="47" t="str">
-        <x:v>activity_register.xml, User.java</x:v>
+        <x:v>activity_post_detail.xml, ChatActivity.java, PanoramaViewActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="107.421875" hidden="0" customHeight="1">
@@ -1109,16 +1115,16 @@
         <x:v>Java/Activity</x:v>
       </x:c>
       <x:c r="C19" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/activities/WelcomeActivity.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/activities/RegisterActivity.java</x:v>
       </x:c>
       <x:c r="D19" s="47" t="str">
-        <x:v>Màn hình chào đầu tiên.</x:v>
+        <x:v>Màn hình đăng ký tài khoản mới.</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Điểm vào điều hướng sang đăng nhập hoặc đăng ký.</x:v>
+        <x:v>Tạo user Firebase Auth và hồ sơ user trên Firestore.</x:v>
       </x:c>
       <x:c r="F19" s="47" t="str">
-        <x:v>activity_welcome.xml, LoginActivity.java, RegisterActivity.java</x:v>
+        <x:v>activity_register.xml, User.java</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="107.421875" hidden="0" customHeight="1">
@@ -1126,22 +1132,22 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B20" s="47" t="str">
-        <x:v>Java/Adapter</x:v>
+        <x:v>Java/Activity</x:v>
       </x:c>
       <x:c r="C20" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/adapters/AdminPostAdapter.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/activities/WelcomeActivity.java</x:v>
       </x:c>
       <x:c r="D20" s="47" t="str">
-        <x:v>Adapter hiển thị danh sách bài cho màn quản trị.</x:v>
+        <x:v>Màn hình chào đầu tiên.</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Bind dữ liệu bài đăng vào item admin để kiểm duyệt/xử lý.</x:v>
+        <x:v>Điểm vào điều hướng sang đăng nhập hoặc đăng ký.</x:v>
       </x:c>
       <x:c r="F20" s="47" t="str">
-        <x:v>item_admin_post.xml, Post.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="120.849609375" hidden="0" customHeight="1">
+        <x:v>activity_welcome.xml, LoginActivity.java, RegisterActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A21" s="50" t="n">
         <x:v>20</x:v>
       </x:c>
@@ -1149,19 +1155,19 @@
         <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C21" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/adapters/ConversationAdapter.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/AdminPostAdapter.java</x:v>
       </x:c>
       <x:c r="D21" s="47" t="str">
-        <x:v>Adapter hiển thị danh sách hội thoại.</x:v>
+        <x:v>Adapter hiển thị danh sách bài cho màn quản trị.</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Bind tên người chat, tin nhắn cuối, thời gian và badge unread.</x:v>
+        <x:v>Bind dữ liệu bài đăng vào item admin để kiểm duyệt/xử lý.</x:v>
       </x:c>
       <x:c r="F21" s="47" t="str">
-        <x:v>item_conversation.xml, Conversation.java, ChatActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>item_admin_post.xml, Post.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="120.849609375" hidden="0" customHeight="1">
       <x:c r="A22" s="50" t="n">
         <x:v>21</x:v>
       </x:c>
@@ -1169,19 +1175,19 @@
         <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C22" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/adapters/MessageAdapter.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/ConversationAdapter.java</x:v>
       </x:c>
       <x:c r="D22" s="47" t="str">
-        <x:v>Adapter hiển thị bubble tin nhắn.</x:v>
+        <x:v>Adapter hiển thị danh sách hội thoại.</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Phân biệt tin gửi/tin nhận, trạng thái đã đọc và nền bubble.</x:v>
+        <x:v>Bind tên người chat, tin nhắn cuối, thời gian và badge unread.</x:v>
       </x:c>
       <x:c r="F22" s="47" t="str">
-        <x:v>item_message.xml, Message.java, ChatActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>item_conversation.xml, Conversation.java, ChatActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="120.849609375" hidden="0" customHeight="1">
       <x:c r="A23" s="50" t="n">
         <x:v>22</x:v>
       </x:c>
@@ -1189,16 +1195,16 @@
         <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C23" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/adapters/PostAdapter.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/MediaPreviewAdapter.java</x:v>
       </x:c>
       <x:c r="D23" s="47" t="str">
-        <x:v>Adapter hiển thị danh sách bài đăng cho người dùng.</x:v>
+        <x:v>Adapter preview ảnh ngang.</x:v>
       </x:c>
       <x:c r="E23" s="47" t="str">
-        <x:v>Bind ảnh, giá, địa chỉ, loại phòng và trạng thái bài.</x:v>
+        <x:v>Hiển thị ảnh đã chọn hoặc ảnh xem trước khi tạo bài.</x:v>
       </x:c>
       <x:c r="F23" s="47" t="str">
-        <x:v>item_post.xml, Post.java, PostDetailActivity.java</x:v>
+        <x:v>item_media_preview.xml, CreatePostActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="107.421875" hidden="0" customHeight="1">
@@ -1209,16 +1215,16 @@
         <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C24" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/adapters/UserAdminAdapter.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/MessageAdapter.java</x:v>
       </x:c>
       <x:c r="D24" s="47" t="str">
-        <x:v>Adapter hiển thị user ở màn admin.</x:v>
+        <x:v>Adapter hiển thị bubble tin nhắn.</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Bind thông tin người dùng và thao tác quản trị liên quan.</x:v>
+        <x:v>Phân biệt tin gửi/tin nhận, trạng thái đã đọc và nền bubble.</x:v>
       </x:c>
       <x:c r="F24" s="47" t="str">
-        <x:v>item_admin_user.xml, User.java</x:v>
+        <x:v>item_message.xml, Message.java, ChatActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="107.421875" hidden="0" customHeight="1">
@@ -1226,59 +1232,59 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B25" s="47" t="str">
-        <x:v>Java/Fragment</x:v>
+        <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C25" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/fragments/HomeFragment.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/PostAdapter.java</x:v>
       </x:c>
       <x:c r="D25" s="47" t="str">
-        <x:v>Fragment trang chủ bài đăng.</x:v>
+        <x:v>Adapter hiển thị danh sách bài đăng cho người dùng.</x:v>
       </x:c>
       <x:c r="E25" s="47" t="str">
-        <x:v>Tìm kiếm, mở bộ lọc ẩn/hiện, lọc bài và sắp xếp theo nhiều tiêu chí.</x:v>
+        <x:v>Bind ảnh, giá, địa chỉ, loại phòng và trạng thái bài.</x:v>
       </x:c>
       <x:c r="F25" s="47" t="str">
-        <x:v>fragment_home.xml, PostAdapter.java, Post.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="120.849609375" hidden="0" customHeight="1">
+        <x:v>item_post.xml, Post.java, PostDetailActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A26" s="50" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="B26" s="47" t="str">
-        <x:v>Java/Fragment</x:v>
+        <x:v>Java/Adapter</x:v>
       </x:c>
       <x:c r="C26" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/fragments/MapFragment.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/adapters/UserAdminAdapter.java</x:v>
       </x:c>
       <x:c r="D26" s="47" t="str">
-        <x:v>Fragment bản đồ Google Maps.</x:v>
+        <x:v>Adapter hiển thị user ở màn admin.</x:v>
       </x:c>
       <x:c r="E26" s="47" t="str">
-        <x:v>Hiển thị bài có tọa độ, ưu tiên bài gần người dùng và làm mờ vị trí bài ở ghép.</x:v>
+        <x:v>Bind thông tin người dùng và thao tác quản trị liên quan.</x:v>
       </x:c>
       <x:c r="F26" s="47" t="str">
-        <x:v>fragment_map.xml, Post.java, PostDetailActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>item_admin_user.xml, User.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A27" s="50" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="B27" s="47" t="str">
-        <x:v>Java/Fragment</x:v>
+        <x:v>Java/Application</x:v>
       </x:c>
       <x:c r="C27" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/fragments/MessagesFragment.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/BTLApplication.java</x:v>
       </x:c>
       <x:c r="D27" s="47" t="str">
-        <x:v>Fragment danh sách hội thoại.</x:v>
+        <x:v>Application class của app.</x:v>
       </x:c>
       <x:c r="E27" s="47" t="str">
-        <x:v>Nghe thay đổi conversation realtime và mở ChatActivity.</x:v>
+        <x:v>Khởi tạo theme đã lưu ngay khi app mở.</x:v>
       </x:c>
       <x:c r="F27" s="47" t="str">
-        <x:v>fragment_messages.xml, ConversationAdapter.java</x:v>
+        <x:v>ThemePreferences.java, MainActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="134.27734375" hidden="0" customHeight="1">
@@ -1289,74 +1295,76 @@
         <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="C28" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/fragments/ProfileFragment.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/fragments/AdminFragment.java</x:v>
       </x:c>
       <x:c r="D28" s="47" t="str">
-        <x:v>Fragment hồ sơ cá nhân.</x:v>
+        <x:v>Fragment tổng hợp công cụ quản trị.</x:v>
       </x:c>
       <x:c r="E28" s="47" t="str">
-        <x:v>Hiển thị thông tin user, điều khiển theme, mở sửa hồ sơ, đăng tin và đăng xuất.</x:v>
+        <x:v>Điểm truy cập các màn quản lý user và bài đăng cho admin.</x:v>
       </x:c>
       <x:c r="F28" s="47" t="str">
-        <x:v>fragment_profile.xml, EditProfileActivity.java, ThemePreferences.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>fragment_admin.xml, AdminUserManagementActivity.java, AdminUserPostsActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A29" s="50" t="n">
         <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="47" t="str">
-        <x:v>Khác</x:v>
+        <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="C29" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/google-services.json</x:v>
+        <x:v>app/src/main/java/com/example/btland/fragments/HomeFragment.java</x:v>
       </x:c>
       <x:c r="D29" s="47" t="str">
-        <x:v>Tệp google-services.</x:v>
+        <x:v>Fragment trang chủ bài đăng.</x:v>
       </x:c>
       <x:c r="E29" s="47" t="str">
-        <x:v>Tài nguyên hoặc cấu hình hỗ trợ cho dự án.</x:v>
-      </x:c>
-      <x:c r="F29" s="47" t="str"/>
-    </x:row>
-    <x:row r="30" ht="147.705078125" hidden="0" customHeight="1">
+        <x:v>Tìm kiếm, mở bộ lọc ẩn/hiện, lọc bài và sắp xếp theo nhiều tiêu chí.</x:v>
+      </x:c>
+      <x:c r="F29" s="47" t="str">
+        <x:v>fragment_home.xml, PostAdapter.java, Post.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="120.849609375" hidden="0" customHeight="1">
       <x:c r="A30" s="50" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="B30" s="47" t="str">
-        <x:v>Java/Model</x:v>
+        <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="C30" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/models/Conversation.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/fragments/MapFragment.java</x:v>
       </x:c>
       <x:c r="D30" s="47" t="str">
-        <x:v>Model dữ liệu cho conversation.</x:v>
+        <x:v>Fragment bản đồ Google Maps.</x:v>
       </x:c>
       <x:c r="E30" s="47" t="str">
-        <x:v>Lưu id hội thoại, userIds, lastMessage, lastTimestamp, unreadCounts và participantNames.</x:v>
+        <x:v>Hiển thị bài có tọa độ, ưu tiên bài gần người dùng và làm mờ vị trí bài ở ghép.</x:v>
       </x:c>
       <x:c r="F30" s="47" t="str">
-        <x:v>ChatActivity.java, MessagesFragment.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>fragment_map.xml, Post.java, PostDetailActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A31" s="50" t="n">
         <x:v>30</x:v>
       </x:c>
       <x:c r="B31" s="47" t="str">
-        <x:v>Java/Model</x:v>
+        <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="C31" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/models/Message.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/fragments/MessagesFragment.java</x:v>
       </x:c>
       <x:c r="D31" s="47" t="str">
-        <x:v>Model dữ liệu cho message.</x:v>
+        <x:v>Fragment danh sách hội thoại.</x:v>
       </x:c>
       <x:c r="E31" s="47" t="str">
-        <x:v>Lưu sender, receiver, nội dung, thời gian và trạng thái read.</x:v>
+        <x:v>Nghe thay đổi conversation realtime và mở ChatActivity.</x:v>
       </x:c>
       <x:c r="F31" s="47" t="str">
-        <x:v>ChatActivity.java, MessageAdapter.java</x:v>
+        <x:v>fragment_messages.xml, ConversationAdapter.java</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="134.27734375" hidden="0" customHeight="1">
@@ -1364,22 +1372,22 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B32" s="47" t="str">
-        <x:v>Java/Model</x:v>
+        <x:v>Java/Fragment</x:v>
       </x:c>
       <x:c r="C32" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/models/Post.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/fragments/ProfileFragment.java</x:v>
       </x:c>
       <x:c r="D32" s="47" t="str">
-        <x:v>Model dữ liệu bài đăng.</x:v>
+        <x:v>Fragment hồ sơ cá nhân.</x:v>
       </x:c>
       <x:c r="E32" s="47" t="str">
-        <x:v>Chứa thông tin mô tả bài, giá, diện tích, GPS, ảnh, panorama và trạng thái hiển thị.</x:v>
+        <x:v>Hiển thị thông tin user, điều khiển theme, mở sửa hồ sơ, đăng tin và đăng xuất.</x:v>
       </x:c>
       <x:c r="F32" s="47" t="str">
-        <x:v>CreatePostActivity.java, PostAdapter.java, MapFragment.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="134.27734375" hidden="0" customHeight="1">
+        <x:v>fragment_profile.xml, EditProfileActivity.java, ThemePreferences.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="147.705078125" hidden="0" customHeight="1">
       <x:c r="A33" s="50" t="n">
         <x:v>32</x:v>
       </x:c>
@@ -1387,96 +1395,96 @@
         <x:v>Java/Model</x:v>
       </x:c>
       <x:c r="C33" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/models/User.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/models/Conversation.java</x:v>
       </x:c>
       <x:c r="D33" s="47" t="str">
-        <x:v>Model dữ liệu người dùng.</x:v>
+        <x:v>Model dữ liệu cho conversation.</x:v>
       </x:c>
       <x:c r="E33" s="47" t="str">
-        <x:v>Chứa thông tin hồ sơ, vai trò admin, trạng thái khóa và avatar.</x:v>
+        <x:v>Lưu id hội thoại, userIds, lastMessage, lastTimestamp, unreadCounts và participantNames.</x:v>
       </x:c>
       <x:c r="F33" s="47" t="str">
-        <x:v>RegisterActivity.java, EditProfileActivity.java, AdminUserManagementActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>ChatActivity.java, MessagesFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A34" s="50" t="n">
         <x:v>33</x:v>
       </x:c>
       <x:c r="B34" s="47" t="str">
-        <x:v>Java/Utility</x:v>
+        <x:v>Java/Model</x:v>
       </x:c>
       <x:c r="C34" s="47" t="str">
-        <x:v>app/src/main/java/com/example/btland/utils/CloudinaryHelper.java</x:v>
+        <x:v>app/src/main/java/com/example/btland/models/Message.java</x:v>
       </x:c>
       <x:c r="D34" s="47" t="str">
-        <x:v>Lớp tiện ích Cloudinary.</x:v>
+        <x:v>Model dữ liệu cho message.</x:v>
       </x:c>
       <x:c r="E34" s="47" t="str">
-        <x:v>Tách logic dùng chung ra khỏi Activity/Fragment để dễ tái sử dụng.</x:v>
+        <x:v>Lưu sender, receiver, nội dung, thời gian và trạng thái read.</x:v>
       </x:c>
       <x:c r="F34" s="47" t="str">
-        <x:v>activities/, fragments/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>ChatActivity.java, MessageAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="134.27734375" hidden="0" customHeight="1">
       <x:c r="A35" s="50" t="n">
         <x:v>34</x:v>
       </x:c>
       <x:c r="B35" s="47" t="str">
-        <x:v>Resource/Drawable</x:v>
+        <x:v>Java/Model</x:v>
       </x:c>
       <x:c r="C35" s="47" t="str">
-        <x:v>app/src/main/res/drawable/ic_launcher_background.xml</x:v>
+        <x:v>app/src/main/java/com/example/btland/models/Post.java</x:v>
       </x:c>
       <x:c r="D35" s="47" t="str">
-        <x:v>Icon vector Launcher Background.</x:v>
+        <x:v>Model dữ liệu bài đăng.</x:v>
       </x:c>
       <x:c r="E35" s="47" t="str">
-        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
+        <x:v>Chứa thông tin mô tả bài, giá, diện tích, GPS, ảnh, panorama và trạng thái hiển thị.</x:v>
       </x:c>
       <x:c r="F35" s="47" t="str">
-        <x:v>layout/*.xml, menu/*.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>CreatePostActivity.java, PostAdapter.java, MapFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="134.27734375" hidden="0" customHeight="1">
       <x:c r="A36" s="50" t="n">
         <x:v>35</x:v>
       </x:c>
       <x:c r="B36" s="47" t="str">
-        <x:v>Resource/Drawable</x:v>
+        <x:v>Java/Model</x:v>
       </x:c>
       <x:c r="C36" s="47" t="str">
-        <x:v>app/src/main/res/drawable/ic_launcher_foreground.xml</x:v>
+        <x:v>app/src/main/java/com/example/btland/models/User.java</x:v>
       </x:c>
       <x:c r="D36" s="47" t="str">
-        <x:v>Icon vector Launcher Foreground.</x:v>
+        <x:v>Model dữ liệu người dùng.</x:v>
       </x:c>
       <x:c r="E36" s="47" t="str">
-        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
+        <x:v>Chứa thông tin hồ sơ, vai trò admin, trạng thái khóa và avatar.</x:v>
       </x:c>
       <x:c r="F36" s="47" t="str">
-        <x:v>layout/*.xml, menu/*.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>RegisterActivity.java, EditProfileActivity.java, AdminUserManagementActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="120.849609375" hidden="0" customHeight="1">
       <x:c r="A37" s="50" t="n">
         <x:v>36</x:v>
       </x:c>
       <x:c r="B37" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Java/Utility</x:v>
       </x:c>
       <x:c r="C37" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_admin_user_management.xml</x:v>
+        <x:v>app/src/main/java/com/example/btland/utils/FirebaseStorageHelper.java</x:v>
       </x:c>
       <x:c r="D37" s="47" t="str">
-        <x:v>Bố cục XML cho màn hình Admin User Management.</x:v>
+        <x:v>Tiện ích thao tác Firebase Storage.</x:v>
       </x:c>
       <x:c r="E37" s="47" t="str">
-        <x:v>Định nghĩa cây view của màn Admin User Management.</x:v>
+        <x:v>Upload file, xóa thư mục và diễn giải lỗi Storage theo ngữ cảnh dễ hiểu.</x:v>
       </x:c>
       <x:c r="F37" s="47" t="str">
-        <x:v>Admin User ManagementActivity.java</x:v>
+        <x:v>CreatePostActivity.java, EditProfileActivity.java, storage.rules</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="93.994140625" hidden="0" customHeight="1">
@@ -1484,59 +1492,59 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B38" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Java/Utility</x:v>
       </x:c>
       <x:c r="C38" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_admin_user_posts.xml</x:v>
+        <x:v>app/src/main/java/com/example/btland/utils/PostRepository.java</x:v>
       </x:c>
       <x:c r="D38" s="47" t="str">
-        <x:v>Bố cục XML cho màn hình Admin User Posts.</x:v>
+        <x:v>Lớp tiện ích thao tác bài đăng.</x:v>
       </x:c>
       <x:c r="E38" s="47" t="str">
-        <x:v>Định nghĩa cây view của màn Admin User Posts.</x:v>
+        <x:v>Đóng gói các thao tác xóa hoặc cập nhật bài để tái sử dụng.</x:v>
       </x:c>
       <x:c r="F38" s="47" t="str">
-        <x:v>Admin User PostsActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>MyPostsActivity.java, Post.java, FirebaseStorageHelper.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="147.705078125" hidden="0" customHeight="1">
       <x:c r="A39" s="50" t="n">
         <x:v>38</x:v>
       </x:c>
       <x:c r="B39" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Java/Utility</x:v>
       </x:c>
       <x:c r="C39" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_chat.xml</x:v>
+        <x:v>app/src/main/java/com/example/btland/utils/ThemePreferences.java</x:v>
       </x:c>
       <x:c r="D39" s="47" t="str">
-        <x:v>Layout màn chat.</x:v>
+        <x:v>Tiện ích lưu thiết lập theme.</x:v>
       </x:c>
       <x:c r="E39" s="47" t="str">
-        <x:v>Sắp xếp tiêu đề hội thoại, danh sách tin nhắn và ô nhập tin.</x:v>
+        <x:v>Lưu mode sáng/tối, auto theme và mode đã áp lần cuối bằng SharedPreferences.</x:v>
       </x:c>
       <x:c r="F39" s="47" t="str">
-        <x:v>ChatActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="134.27734375" hidden="0" customHeight="1">
+        <x:v>BTLApplication.java, MainActivity.java, ProfileFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A40" s="50" t="n">
         <x:v>39</x:v>
       </x:c>
       <x:c r="B40" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Color</x:v>
       </x:c>
       <x:c r="C40" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_create_post.xml</x:v>
+        <x:v>app/src/main/res/color/bottom_nav_item_color.xml</x:v>
       </x:c>
       <x:c r="D40" s="47" t="str">
-        <x:v>Layout màn tạo bài đăng.</x:v>
+        <x:v>Color selector Bottom Nav Item Color.</x:v>
       </x:c>
       <x:c r="E40" s="47" t="str">
-        <x:v>Chứa form nhập bài, khu chọn ảnh, nút tạo panorama và preview bài.</x:v>
+        <x:v>Điều khiển màu động theo trạng thái selected/checked.</x:v>
       </x:c>
       <x:c r="F40" s="47" t="str">
-        <x:v>CreatePostActivity.java</x:v>
+        <x:v>activity_main.xml, menu/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="80.56640625" hidden="0" customHeight="1">
@@ -1544,59 +1552,59 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B41" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C41" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_edit_post.xml</x:v>
+        <x:v>app/src/main/res/drawable/bg_badge_unread.xml</x:v>
       </x:c>
       <x:c r="D41" s="47" t="str">
-        <x:v>Layout màn sửa bài đăng.</x:v>
+        <x:v>Shape/background Badge Unread.</x:v>
       </x:c>
       <x:c r="E41" s="47" t="str">
-        <x:v>Hiển thị form chỉnh sửa nội dung bài hiện có.</x:v>
+        <x:v>Cung cấp nền, bo góc, viền hoặc badge cho UI.</x:v>
       </x:c>
       <x:c r="F41" s="47" t="str">
-        <x:v>EditPostActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>layout/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A42" s="50" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C42" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_edit_profile.xml</x:v>
+        <x:v>app/src/main/res/drawable/bg_map_overlay.xml</x:v>
       </x:c>
       <x:c r="D42" s="47" t="str">
-        <x:v>Layout màn sửa hồ sơ.</x:v>
+        <x:v>Shape/background Map Overlay.</x:v>
       </x:c>
       <x:c r="E42" s="47" t="str">
-        <x:v>Hiển thị avatar, tên, số điện thoại và nút lưu hồ sơ.</x:v>
+        <x:v>Cung cấp nền, bo góc, viền hoặc badge cho UI.</x:v>
       </x:c>
       <x:c r="F42" s="47" t="str">
-        <x:v>EditProfileActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="67.138671875" hidden="0" customHeight="1">
+        <x:v>layout/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A43" s="50" t="n">
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C43" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_login.xml</x:v>
+        <x:v>app/src/main/res/drawable/bg_message_incoming.xml</x:v>
       </x:c>
       <x:c r="D43" s="47" t="str">
-        <x:v>Layout màn đăng nhập.</x:v>
+        <x:v>Shape/background Message Incoming.</x:v>
       </x:c>
       <x:c r="E43" s="47" t="str">
-        <x:v>Hiển thị ô email/mật khẩu và nút đăng nhập.</x:v>
+        <x:v>Cung cấp nền, bo góc, viền hoặc badge cho UI.</x:v>
       </x:c>
       <x:c r="F43" s="47" t="str">
-        <x:v>LoginActivity.java</x:v>
+        <x:v>layout/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="80.56640625" hidden="0" customHeight="1">
@@ -1604,19 +1612,19 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C44" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_main.xml</x:v>
+        <x:v>app/src/main/res/drawable/bg_message_outgoing.xml</x:v>
       </x:c>
       <x:c r="D44" s="47" t="str">
-        <x:v>Layout khung chính của app.</x:v>
+        <x:v>Shape/background Message Outgoing.</x:v>
       </x:c>
       <x:c r="E44" s="47" t="str">
-        <x:v>Chứa FrameLayout và BottomNavigationView.</x:v>
+        <x:v>Cung cấp nền, bo góc, viền hoặc badge cho UI.</x:v>
       </x:c>
       <x:c r="F44" s="47" t="str">
-        <x:v>MainActivity.java, bottom_nav_menu.xml</x:v>
+        <x:v>layout/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="80.56640625" hidden="0" customHeight="1">
@@ -1624,19 +1632,19 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C45" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_my_posts.xml</x:v>
+        <x:v>app/src/main/res/drawable/bg_round_button.xml</x:v>
       </x:c>
       <x:c r="D45" s="47" t="str">
-        <x:v>Layout màn bài đăng của tôi.</x:v>
+        <x:v>Shape/background Round Button.</x:v>
       </x:c>
       <x:c r="E45" s="47" t="str">
-        <x:v>Hiển thị danh sách bài thuộc user hiện tại.</x:v>
+        <x:v>Cung cấp nền, bo góc, viền hoặc badge cho UI.</x:v>
       </x:c>
       <x:c r="F45" s="47" t="str">
-        <x:v>MyPostsActivity.java, PostAdapter.java</x:v>
+        <x:v>layout/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="93.994140625" hidden="0" customHeight="1">
@@ -1644,39 +1652,39 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C46" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_post_detail.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_close.xml</x:v>
       </x:c>
       <x:c r="D46" s="47" t="str">
-        <x:v>Layout màn chi tiết bài đăng.</x:v>
+        <x:v>Icon vector Close.</x:v>
       </x:c>
       <x:c r="E46" s="47" t="str">
-        <x:v>Hiển thị thông tin bài, ảnh, nút chat và panorama.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F46" s="47" t="str">
-        <x:v>PostDetailActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="67.138671875" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A47" s="50" t="n">
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C47" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_register.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_filter_list.xml</x:v>
       </x:c>
       <x:c r="D47" s="47" t="str">
-        <x:v>Layout màn đăng ký.</x:v>
+        <x:v>Icon vector Filter List.</x:v>
       </x:c>
       <x:c r="E47" s="47" t="str">
-        <x:v>Hiển thị form tạo tài khoản mới.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F47" s="47" t="str">
-        <x:v>RegisterActivity.java</x:v>
+        <x:v>layout/*.xml, menu/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="93.994140625" hidden="0" customHeight="1">
@@ -1684,59 +1692,59 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C48" s="47" t="str">
-        <x:v>app/src/main/res/layout/activity_welcome.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_launcher_background.xml</x:v>
       </x:c>
       <x:c r="D48" s="47" t="str">
-        <x:v>Layout màn chào.</x:v>
+        <x:v>Icon vector Launcher Background.</x:v>
       </x:c>
       <x:c r="E48" s="47" t="str">
-        <x:v>Hiển thị lựa chọn đi tới đăng nhập hoặc đăng ký.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F48" s="47" t="str">
-        <x:v>WelcomeActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="134.27734375" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A49" s="50" t="n">
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C49" s="47" t="str">
-        <x:v>app/src/main/res/layout/fragment_home.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_launcher_foreground.xml</x:v>
       </x:c>
       <x:c r="D49" s="47" t="str">
-        <x:v>Layout fragment trang chủ.</x:v>
+        <x:v>Icon vector Launcher Foreground.</x:v>
       </x:c>
       <x:c r="E49" s="47" t="str">
-        <x:v>Chứa thanh tìm kiếm, filter panel cuộn riêng và danh sách bài đăng.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F49" s="47" t="str">
-        <x:v>HomeFragment.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A50" s="50" t="n">
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C50" s="47" t="str">
-        <x:v>app/src/main/res/layout/fragment_map.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_my_location.xml</x:v>
       </x:c>
       <x:c r="D50" s="47" t="str">
-        <x:v>Layout fragment bản đồ.</x:v>
+        <x:v>Icon vector My Location.</x:v>
       </x:c>
       <x:c r="E50" s="47" t="str">
-        <x:v>Chứa MapView, trạng thái bản đồ và nút lấy lại GPS.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F50" s="47" t="str">
-        <x:v>MapFragment.java</x:v>
+        <x:v>layout/*.xml, menu/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="93.994140625" hidden="0" customHeight="1">
@@ -1744,79 +1752,79 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C51" s="47" t="str">
-        <x:v>app/src/main/res/layout/fragment_messages.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_nav_admin.xml</x:v>
       </x:c>
       <x:c r="D51" s="47" t="str">
-        <x:v>Layout fragment hội thoại.</x:v>
+        <x:v>Icon vector Nav Admin.</x:v>
       </x:c>
       <x:c r="E51" s="47" t="str">
-        <x:v>Hiển thị danh sách conversation và trạng thái rỗng.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F51" s="47" t="str">
-        <x:v>MessagesFragment.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A52" s="50" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C52" s="47" t="str">
-        <x:v>app/src/main/res/layout/fragment_profile.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_nav_home.xml</x:v>
       </x:c>
       <x:c r="D52" s="47" t="str">
-        <x:v>Layout fragment hồ sơ.</x:v>
+        <x:v>Icon vector Nav Home.</x:v>
       </x:c>
       <x:c r="E52" s="47" t="str">
-        <x:v>Hiển thị thông tin user, điều khiển theme và các nút thao tác cá nhân.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F52" s="47" t="str">
-        <x:v>ProfileFragment.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A53" s="50" t="n">
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C53" s="47" t="str">
-        <x:v>app/src/main/res/layout/item_admin_post.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_nav_map.xml</x:v>
       </x:c>
       <x:c r="D53" s="47" t="str">
-        <x:v>Layout item bài đăng cho admin.</x:v>
+        <x:v>Icon vector Nav Map.</x:v>
       </x:c>
       <x:c r="E53" s="47" t="str">
-        <x:v>Card con dùng trong danh sách kiểm duyệt bài.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F53" s="47" t="str">
-        <x:v>AdminPostAdapter.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A54" s="50" t="n">
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C54" s="47" t="str">
-        <x:v>app/src/main/res/layout/item_admin_user.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_nav_messages.xml</x:v>
       </x:c>
       <x:c r="D54" s="47" t="str">
-        <x:v>Layout item user cho admin.</x:v>
+        <x:v>Icon vector Nav Messages.</x:v>
       </x:c>
       <x:c r="E54" s="47" t="str">
-        <x:v>Card con dùng trong danh sách quản lý người dùng.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F54" s="47" t="str">
-        <x:v>UserAdminAdapter.java</x:v>
+        <x:v>layout/*.xml, menu/*.xml</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="93.994140625" hidden="0" customHeight="1">
@@ -1824,42 +1832,42 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C55" s="47" t="str">
-        <x:v>app/src/main/res/layout/item_conversation.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_nav_profile.xml</x:v>
       </x:c>
       <x:c r="D55" s="47" t="str">
-        <x:v>Layout item hội thoại.</x:v>
+        <x:v>Icon vector Nav Profile.</x:v>
       </x:c>
       <x:c r="E55" s="47" t="str">
-        <x:v>Card con hiển thị người chat, tin cuối và badge unread.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F55" s="47" t="str">
-        <x:v>ConversationAdapter.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A56" s="50" t="n">
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" s="47" t="str">
-        <x:v>Resource/Layout</x:v>
+        <x:v>Resource/Drawable</x:v>
       </x:c>
       <x:c r="C56" s="47" t="str">
-        <x:v>app/src/main/res/layout/item_message.xml</x:v>
+        <x:v>app/src/main/res/drawable/ic_search.xml</x:v>
       </x:c>
       <x:c r="D56" s="47" t="str">
-        <x:v>Layout item tin nhắn.</x:v>
+        <x:v>Icon vector Search.</x:v>
       </x:c>
       <x:c r="E56" s="47" t="str">
-        <x:v>Khung bubble tin nhắn cho message gửi/nhận.</x:v>
+        <x:v>Cung cấp icon hiển thị cho nút, nav hoặc trạng thái.</x:v>
       </x:c>
       <x:c r="F56" s="47" t="str">
-        <x:v>MessageAdapter.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>layout/*.xml, menu/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A57" s="50" t="n">
         <x:v>56</x:v>
       </x:c>
@@ -1867,36 +1875,36 @@
         <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C57" s="47" t="str">
-        <x:v>app/src/main/res/layout/item_post.xml</x:v>
+        <x:v>app/src/main/res/layout/activity_admin_user_management.xml</x:v>
       </x:c>
       <x:c r="D57" s="47" t="str">
-        <x:v>Layout item bài đăng.</x:v>
+        <x:v>Bố cục XML cho màn hình Admin User Management.</x:v>
       </x:c>
       <x:c r="E57" s="47" t="str">
-        <x:v>Card bài đăng hiển thị ảnh đại diện và thông tin tóm tắt.</x:v>
+        <x:v>Định nghĩa cây view của màn Admin User Management.</x:v>
       </x:c>
       <x:c r="F57" s="47" t="str">
-        <x:v>PostAdapter.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="107.421875" hidden="0" customHeight="1">
+        <x:v>Admin User ManagementActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A58" s="50" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" s="47" t="str">
-        <x:v>Resource/Menu</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C58" s="47" t="str">
-        <x:v>app/src/main/res/menu/bottom_nav_menu.xml</x:v>
+        <x:v>app/src/main/res/layout/activity_admin_user_posts.xml</x:v>
       </x:c>
       <x:c r="D58" s="47" t="str">
-        <x:v>Menu Bottom Navigation.</x:v>
+        <x:v>Bố cục XML cho màn hình Admin User Posts.</x:v>
       </x:c>
       <x:c r="E58" s="47" t="str">
-        <x:v>Định nghĩa các tab Trang chủ, Bản đồ, Tin nhắn, Cá nhân và Quản trị.</x:v>
+        <x:v>Định nghĩa cây view của màn Admin User Posts.</x:v>
       </x:c>
       <x:c r="F58" s="47" t="str">
-        <x:v>activity_main.xml, MainActivity.java</x:v>
+        <x:v>Admin User PostsActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="93.994140625" hidden="0" customHeight="1">
@@ -1904,99 +1912,99 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C59" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-anydpi-v26/ic_launcher_round.xml</x:v>
+        <x:v>app/src/main/res/layout/activity_chat.xml</x:v>
       </x:c>
       <x:c r="D59" s="47" t="str">
-        <x:v>Launcher icon density mipmap-anydpi-v26.</x:v>
+        <x:v>Layout màn chat.</x:v>
       </x:c>
       <x:c r="E59" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Sắp xếp tiêu đề hội thoại, danh sách tin nhắn và ô nhập tin.</x:v>
       </x:c>
       <x:c r="F59" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>ChatActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="134.27734375" hidden="0" customHeight="1">
       <x:c r="A60" s="50" t="n">
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C60" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-anydpi-v26/ic_launcher.xml</x:v>
+        <x:v>app/src/main/res/layout/activity_create_post.xml</x:v>
       </x:c>
       <x:c r="D60" s="47" t="str">
-        <x:v>Launcher icon density mipmap-anydpi-v26.</x:v>
+        <x:v>Layout màn tạo bài đăng.</x:v>
       </x:c>
       <x:c r="E60" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Chứa form nhập bài, khu chọn ảnh, nút chọn ảnh 360 và phần preview bài.</x:v>
       </x:c>
       <x:c r="F60" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>CreatePostActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A61" s="50" t="n">
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C61" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-hdpi/ic_launcher_round.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_edit_post.xml</x:v>
       </x:c>
       <x:c r="D61" s="47" t="str">
-        <x:v>Launcher icon density mipmap-hdpi.</x:v>
+        <x:v>Layout màn sửa bài đăng.</x:v>
       </x:c>
       <x:c r="E61" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị form chỉnh sửa nội dung bài hiện có.</x:v>
       </x:c>
       <x:c r="F61" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>EditPostActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A62" s="50" t="n">
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C62" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-hdpi/ic_launcher.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_edit_profile.xml</x:v>
       </x:c>
       <x:c r="D62" s="47" t="str">
-        <x:v>Launcher icon density mipmap-hdpi.</x:v>
+        <x:v>Layout màn sửa hồ sơ.</x:v>
       </x:c>
       <x:c r="E62" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị avatar, tên, số điện thoại và nút lưu hồ sơ.</x:v>
       </x:c>
       <x:c r="F62" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>EditProfileActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="67.138671875" hidden="0" customHeight="1">
       <x:c r="A63" s="50" t="n">
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C63" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-mdpi/ic_launcher_round.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_login.xml</x:v>
       </x:c>
       <x:c r="D63" s="47" t="str">
-        <x:v>Launcher icon density mipmap-mdpi.</x:v>
+        <x:v>Layout màn đăng nhập.</x:v>
       </x:c>
       <x:c r="E63" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị ô email/mật khẩu và nút đăng nhập.</x:v>
       </x:c>
       <x:c r="F63" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>LoginActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="80.56640625" hidden="0" customHeight="1">
@@ -2004,59 +2012,59 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C64" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-mdpi/ic_launcher.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_main.xml</x:v>
       </x:c>
       <x:c r="D64" s="47" t="str">
-        <x:v>Launcher icon density mipmap-mdpi.</x:v>
+        <x:v>Layout khung chính của app.</x:v>
       </x:c>
       <x:c r="E64" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Chứa FrameLayout và BottomNavigationView.</x:v>
       </x:c>
       <x:c r="F64" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>MainActivity.java, bottom_nav_menu.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A65" s="50" t="n">
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C65" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xhdpi/ic_launcher_round.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_my_posts.xml</x:v>
       </x:c>
       <x:c r="D65" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xhdpi.</x:v>
+        <x:v>Layout màn bài đăng của tôi.</x:v>
       </x:c>
       <x:c r="E65" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị danh sách bài thuộc user hiện tại.</x:v>
       </x:c>
       <x:c r="F65" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>MyPostsActivity.java, PostAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A66" s="50" t="n">
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C66" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xhdpi/ic_launcher.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_panorama_view.xml</x:v>
       </x:c>
       <x:c r="D66" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xhdpi.</x:v>
+        <x:v>Layout màn xem panorama.</x:v>
       </x:c>
       <x:c r="E66" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Chứa vùng cuộn ngang và hint điều khiển ảnh 360.</x:v>
       </x:c>
       <x:c r="F66" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>PanoramaViewActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="93.994140625" hidden="0" customHeight="1">
@@ -2064,39 +2072,39 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C67" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xxhdpi/ic_launcher_round.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_post_detail.xml</x:v>
       </x:c>
       <x:c r="D67" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xxhdpi.</x:v>
+        <x:v>Layout màn chi tiết bài đăng.</x:v>
       </x:c>
       <x:c r="E67" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị thông tin bài, ảnh, nút chat và panorama.</x:v>
       </x:c>
       <x:c r="F67" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>PostDetailActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="67.138671875" hidden="0" customHeight="1">
       <x:c r="A68" s="50" t="n">
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C68" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xxhdpi/ic_launcher.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_register.xml</x:v>
       </x:c>
       <x:c r="D68" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xxhdpi.</x:v>
+        <x:v>Layout màn đăng ký.</x:v>
       </x:c>
       <x:c r="E68" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị form tạo tài khoản mới.</x:v>
       </x:c>
       <x:c r="F68" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>RegisterActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="93.994140625" hidden="0" customHeight="1">
@@ -2104,19 +2112,19 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C69" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xxxhdpi/ic_launcher_round.webp</x:v>
+        <x:v>app/src/main/res/layout/activity_welcome.xml</x:v>
       </x:c>
       <x:c r="D69" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xxxhdpi.</x:v>
+        <x:v>Layout màn chào.</x:v>
       </x:c>
       <x:c r="E69" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Hiển thị lựa chọn đi tới đăng nhập hoặc đăng ký.</x:v>
       </x:c>
       <x:c r="F69" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>WelcomeActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="80.56640625" hidden="0" customHeight="1">
@@ -2124,99 +2132,99 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" s="47" t="str">
-        <x:v>Launcher Asset</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C70" s="47" t="str">
-        <x:v>app/src/main/res/mipmap-xxxhdpi/ic_launcher.webp</x:v>
+        <x:v>app/src/main/res/layout/fragment_admin.xml</x:v>
       </x:c>
       <x:c r="D70" s="47" t="str">
-        <x:v>Launcher icon density mipmap-xxxhdpi.</x:v>
+        <x:v>Layout fragment quản trị.</x:v>
       </x:c>
       <x:c r="E70" s="47" t="str">
-        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+        <x:v>Bố trí các nút hoặc thẻ điều hướng cho admin.</x:v>
       </x:c>
       <x:c r="F70" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="67.138671875" hidden="0" customHeight="1">
+        <x:v>AdminFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="134.27734375" hidden="0" customHeight="1">
       <x:c r="A71" s="50" t="n">
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" s="47" t="str">
-        <x:v>Resource/Value</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C71" s="47" t="str">
-        <x:v>app/src/main/res/values/colors.xml</x:v>
+        <x:v>app/src/main/res/layout/fragment_home.xml</x:v>
       </x:c>
       <x:c r="D71" s="47" t="str">
-        <x:v>Bảng màu dùng toàn app.</x:v>
+        <x:v>Layout fragment trang chủ.</x:v>
       </x:c>
       <x:c r="E71" s="47" t="str">
-        <x:v>Tập trung các mã màu chủ đạo cho UI.</x:v>
+        <x:v>Chứa thanh tìm kiếm, filter panel cuộn riêng và danh sách bài đăng.</x:v>
       </x:c>
       <x:c r="F71" s="47" t="str">
-        <x:v>themes.xml, drawable/bg_*.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>HomeFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A72" s="50" t="n">
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" s="47" t="str">
-        <x:v>Resource/Value</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C72" s="47" t="str">
-        <x:v>app/src/main/res/values/strings.xml</x:v>
+        <x:v>app/src/main/res/layout/fragment_map.xml</x:v>
       </x:c>
       <x:c r="D72" s="47" t="str">
-        <x:v>Kho chuỗi văn bản tổng quát của Android.</x:v>
+        <x:v>Layout fragment bản đồ.</x:v>
       </x:c>
       <x:c r="E72" s="47" t="str">
-        <x:v>Nơi nên đặt string dùng lại nếu cần chuẩn hóa thêm.</x:v>
+        <x:v>Chứa MapView, trạng thái bản đồ và nút lấy lại GPS.</x:v>
       </x:c>
       <x:c r="F72" s="47" t="str">
-        <x:v>layout/*.xml</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="134.27734375" hidden="0" customHeight="1">
+        <x:v>MapFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A73" s="50" t="n">
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" s="47" t="str">
-        <x:v>Resource/Theme</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C73" s="47" t="str">
-        <x:v>app/src/main/res/values/themes.xml</x:v>
+        <x:v>app/src/main/res/layout/fragment_messages.xml</x:v>
       </x:c>
       <x:c r="D73" s="47" t="str">
-        <x:v>Theme sáng và mặc định của ứng dụng.</x:v>
+        <x:v>Layout fragment hội thoại.</x:v>
       </x:c>
       <x:c r="E73" s="47" t="str">
-        <x:v>Quy định màu chủ đạo, status bar, navigation bar và window background.</x:v>
+        <x:v>Hiển thị danh sách conversation và trạng thái rỗng.</x:v>
       </x:c>
       <x:c r="F73" s="47" t="str">
-        <x:v>themes-night/themes.xml, MainActivity.java</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>MessagesFragment.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A74" s="50" t="n">
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" s="47" t="str">
-        <x:v>Resource/XML</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C74" s="47" t="str">
-        <x:v>app/src/main/res/xml/backup_rules.xml</x:v>
+        <x:v>app/src/main/res/layout/fragment_profile.xml</x:v>
       </x:c>
       <x:c r="D74" s="47" t="str">
-        <x:v>Cấu hình auto backup Android.</x:v>
+        <x:v>Layout fragment hồ sơ.</x:v>
       </x:c>
       <x:c r="E74" s="47" t="str">
-        <x:v>Điều khiển phạm vi dữ liệu được backup/restore.</x:v>
+        <x:v>Hiển thị thông tin user, điều khiển theme và các nút thao tác cá nhân.</x:v>
       </x:c>
       <x:c r="F74" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>ProfileFragment.java</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="80.56640625" hidden="0" customHeight="1">
@@ -2224,19 +2232,19 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" s="47" t="str">
-        <x:v>Resource/XML</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C75" s="47" t="str">
-        <x:v>app/src/main/res/xml/data_extraction_rules.xml</x:v>
+        <x:v>app/src/main/res/layout/item_admin_post.xml</x:v>
       </x:c>
       <x:c r="D75" s="47" t="str">
-        <x:v>Cấu hình data extraction cho Android 12+.</x:v>
+        <x:v>Layout item bài đăng cho admin.</x:v>
       </x:c>
       <x:c r="E75" s="47" t="str">
-        <x:v>Kiểm soát dữ liệu cho backup và transfer.</x:v>
+        <x:v>Card con dùng trong danh sách kiểm duyệt bài.</x:v>
       </x:c>
       <x:c r="F75" s="47" t="str">
-        <x:v>AndroidManifest.xml</x:v>
+        <x:v>AdminPostAdapter.java</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="107.421875" hidden="0" customHeight="1">
@@ -2244,119 +2252,119 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" s="47" t="str">
-        <x:v>Cấu hình gốc</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C76" s="47" t="str">
-        <x:v>build.gradle.kts</x:v>
+        <x:v>app/src/main/res/layout/item_admin_user.xml</x:v>
       </x:c>
       <x:c r="D76" s="47" t="str">
-        <x:v>Khai báo pluginManagement và repository dùng cho toàn project.</x:v>
+        <x:v>Layout item user cho admin.</x:v>
       </x:c>
       <x:c r="E76" s="47" t="str">
-        <x:v>Điểm khởi tạo Gradle ở cấp root.</x:v>
+        <x:v>Card con dùng trong danh sách quản lý người dùng.</x:v>
       </x:c>
       <x:c r="F76" s="47" t="str">
-        <x:v>settings.gradle.kts, app/build.gradle.kts</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="77" ht="147.705078125" hidden="0" customHeight="1">
+        <x:v>UserAdminAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A77" s="50" t="n">
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" s="47" t="str">
-        <x:v>Tài liệu</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C77" s="47" t="str">
-        <x:v>FIREBASE_MAPS_SETUP.md</x:v>
+        <x:v>app/src/main/res/layout/item_conversation.xml</x:v>
       </x:c>
       <x:c r="D77" s="47" t="str">
-        <x:v>Tài liệu hướng dẫn cấu hình Firebase Storage, Google Maps, SHA1 và kiểm tra nhanh.</x:v>
+        <x:v>Layout item hội thoại.</x:v>
       </x:c>
       <x:c r="E77" s="47" t="str">
-        <x:v>Giúp đồng bộ console Firebase/Google Cloud với mã nguồn hiện tại.</x:v>
+        <x:v>Card con hiển thị người chat, tin cuối và badge unread.</x:v>
       </x:c>
       <x:c r="F77" s="47" t="str">
-        <x:v>app/src/google-services.json, AndroidManifest.xml, firestore.rules, storage.rules</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="78" ht="147.705078125" hidden="0" customHeight="1">
+        <x:v>ConversationAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A78" s="50" t="n">
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" s="47" t="str">
-        <x:v>Bảo mật Firebase</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C78" s="47" t="str">
-        <x:v>firestore.rules</x:v>
+        <x:v>app/src/main/res/layout/item_media_preview.xml</x:v>
       </x:c>
       <x:c r="D78" s="47" t="str">
-        <x:v>Luật truy cập Firestore cho users, posts, conversations, messages và notifications.</x:v>
+        <x:v>Layout item preview media.</x:v>
       </x:c>
       <x:c r="E78" s="47" t="str">
-        <x:v>Bảo vệ dữ liệu chat, bài đăng và hồ sơ trên Firestore.</x:v>
+        <x:v>Item ảnh nhỏ cho danh sách preview ngang.</x:v>
       </x:c>
       <x:c r="F78" s="47" t="str">
-        <x:v>storage.rules, app/src/google-services.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>MediaPreviewAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A79" s="50" t="n">
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" s="47" t="str">
-        <x:v>Cấu hình gốc</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C79" s="47" t="str">
-        <x:v>gradle.properties</x:v>
+        <x:v>app/src/main/res/layout/item_message.xml</x:v>
       </x:c>
       <x:c r="D79" s="47" t="str">
-        <x:v>Thiết lập JVM args, AndroidX và tối ưu build.</x:v>
+        <x:v>Layout item tin nhắn.</x:v>
       </x:c>
       <x:c r="E79" s="47" t="str">
-        <x:v>Điều chỉnh hành vi Gradle trên máy phát triển.</x:v>
+        <x:v>Khung bubble tin nhắn cho message gửi/nhận.</x:v>
       </x:c>
       <x:c r="F79" s="47" t="str">
-        <x:v>build.gradle.kts</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>MessageAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="93.994140625" hidden="0" customHeight="1">
       <x:c r="A80" s="50" t="n">
         <x:v>79</x:v>
       </x:c>
       <x:c r="B80" s="47" t="str">
-        <x:v>Công cụ build</x:v>
+        <x:v>Resource/Layout</x:v>
       </x:c>
       <x:c r="C80" s="47" t="str">
-        <x:v>gradlew</x:v>
+        <x:v>app/src/main/res/layout/item_post.xml</x:v>
       </x:c>
       <x:c r="D80" s="47" t="str">
-        <x:v>Wrapper script cho Gradle trên Unix/Linux/macOS.</x:v>
+        <x:v>Layout item bài đăng.</x:v>
       </x:c>
       <x:c r="E80" s="47" t="str">
-        <x:v>Cho phép build mà không cần cài Gradle toàn cục.</x:v>
+        <x:v>Card bài đăng hiển thị ảnh đại diện và thông tin tóm tắt.</x:v>
       </x:c>
       <x:c r="F80" s="47" t="str">
-        <x:v>gradlew.bat, gradle/wrapper</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="80.56640625" hidden="0" customHeight="1">
+        <x:v>PostAdapter.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="107.421875" hidden="0" customHeight="1">
       <x:c r="A81" s="50" t="n">
         <x:v>80</x:v>
       </x:c>
       <x:c r="B81" s="47" t="str">
-        <x:v>Công cụ build</x:v>
+        <x:v>Resource/Menu</x:v>
       </x:c>
       <x:c r="C81" s="47" t="str">
-        <x:v>gradlew.bat</x:v>
+        <x:v>app/src/main/res/menu/bottom_nav_menu.xml</x:v>
       </x:c>
       <x:c r="D81" s="47" t="str">
-        <x:v>Wrapper script cho Gradle trên Windows.</x:v>
+        <x:v>Menu Bottom Navigation.</x:v>
       </x:c>
       <x:c r="E81" s="47" t="str">
-        <x:v>Lệnh chuẩn để build dự án trên máy Windows.</x:v>
+        <x:v>Định nghĩa các tab Trang chủ, Bản đồ, Tin nhắn, Cá nhân và Quản trị.</x:v>
       </x:c>
       <x:c r="F81" s="47" t="str">
-        <x:v>gradlew, gradle/wrapper</x:v>
+        <x:v>activity_main.xml, MainActivity.java</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="93.994140625" hidden="0" customHeight="1">
@@ -2364,38 +2372,518 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B82" s="47" t="str">
-        <x:v>Cấu hình gốc</x:v>
+        <x:v>Launcher Asset</x:v>
       </x:c>
       <x:c r="C82" s="47" t="str">
-        <x:v>settings.gradle.kts</x:v>
+        <x:v>app/src/main/res/mipmap-anydpi-v26/ic_launcher_round.xml</x:v>
       </x:c>
       <x:c r="D82" s="47" t="str">
-        <x:v>Đặt tên project BTLAND và include module app.</x:v>
+        <x:v>Launcher icon density mipmap-anydpi-v26.</x:v>
       </x:c>
       <x:c r="E82" s="47" t="str">
-        <x:v>Xác định cấu trúc module mà Gradle sẽ build.</x:v>
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
       </x:c>
       <x:c r="F82" s="47" t="str">
-        <x:v>build.gradle.kts, app/build.gradle.kts</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="93.994140625" hidden="0" customHeight="1">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="80.56640625" hidden="0" customHeight="1">
       <x:c r="A83" s="50" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="B83" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C83" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-anydpi-v26/ic_launcher.xml</x:v>
+      </x:c>
+      <x:c r="D83" s="47" t="str">
+        <x:v>Launcher icon density mipmap-anydpi-v26.</x:v>
+      </x:c>
+      <x:c r="E83" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F83" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A84" s="50" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="B84" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C84" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-hdpi/ic_launcher_round.webp</x:v>
+      </x:c>
+      <x:c r="D84" s="47" t="str">
+        <x:v>Launcher icon density mipmap-hdpi.</x:v>
+      </x:c>
+      <x:c r="E84" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F84" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A85" s="50" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B85" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C85" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-hdpi/ic_launcher.webp</x:v>
+      </x:c>
+      <x:c r="D85" s="47" t="str">
+        <x:v>Launcher icon density mipmap-hdpi.</x:v>
+      </x:c>
+      <x:c r="E85" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F85" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A86" s="50" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="B86" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C86" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-mdpi/ic_launcher_round.webp</x:v>
+      </x:c>
+      <x:c r="D86" s="47" t="str">
+        <x:v>Launcher icon density mipmap-mdpi.</x:v>
+      </x:c>
+      <x:c r="E86" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F86" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A87" s="50" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="B87" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C87" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-mdpi/ic_launcher.webp</x:v>
+      </x:c>
+      <x:c r="D87" s="47" t="str">
+        <x:v>Launcher icon density mipmap-mdpi.</x:v>
+      </x:c>
+      <x:c r="E87" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F87" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A88" s="50" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B88" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C88" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xhdpi/ic_launcher_round.webp</x:v>
+      </x:c>
+      <x:c r="D88" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xhdpi.</x:v>
+      </x:c>
+      <x:c r="E88" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F88" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A89" s="50" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="B89" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C89" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xhdpi/ic_launcher.webp</x:v>
+      </x:c>
+      <x:c r="D89" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xhdpi.</x:v>
+      </x:c>
+      <x:c r="E89" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F89" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A90" s="50" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="B90" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C90" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xxhdpi/ic_launcher_round.webp</x:v>
+      </x:c>
+      <x:c r="D90" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xxhdpi.</x:v>
+      </x:c>
+      <x:c r="E90" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F90" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A91" s="50" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="B91" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C91" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xxhdpi/ic_launcher.webp</x:v>
+      </x:c>
+      <x:c r="D91" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xxhdpi.</x:v>
+      </x:c>
+      <x:c r="E91" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F91" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A92" s="50" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B92" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C92" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xxxhdpi/ic_launcher_round.webp</x:v>
+      </x:c>
+      <x:c r="D92" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xxxhdpi.</x:v>
+      </x:c>
+      <x:c r="E92" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F92" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A93" s="50" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="B93" s="47" t="str">
+        <x:v>Launcher Asset</x:v>
+      </x:c>
+      <x:c r="C93" s="47" t="str">
+        <x:v>app/src/main/res/mipmap-xxxhdpi/ic_launcher.webp</x:v>
+      </x:c>
+      <x:c r="D93" s="47" t="str">
+        <x:v>Launcher icon density mipmap-xxxhdpi.</x:v>
+      </x:c>
+      <x:c r="E93" s="47" t="str">
+        <x:v>Biến thể icon ứng dụng theo từng mật độ màn hình.</x:v>
+      </x:c>
+      <x:c r="F93" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A94" s="50" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="B94" s="47" t="str">
+        <x:v>Resource/Theme</x:v>
+      </x:c>
+      <x:c r="C94" s="47" t="str">
+        <x:v>app/src/main/res/values-night/themes.xml</x:v>
+      </x:c>
+      <x:c r="D94" s="47" t="str">
+        <x:v>Theme tối của ứng dụng.</x:v>
+      </x:c>
+      <x:c r="E94" s="47" t="str">
+        <x:v>Tùy biến giao diện khi app chuyển sang dark mode.</x:v>
+      </x:c>
+      <x:c r="F94" s="47" t="str">
+        <x:v>values/themes.xml, ThemePreferences.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="67.138671875" hidden="0" customHeight="1">
+      <x:c r="A95" s="50" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="B95" s="47" t="str">
+        <x:v>Resource/Value</x:v>
+      </x:c>
+      <x:c r="C95" s="47" t="str">
+        <x:v>app/src/main/res/values/colors.xml</x:v>
+      </x:c>
+      <x:c r="D95" s="47" t="str">
+        <x:v>Bảng màu dùng toàn app.</x:v>
+      </x:c>
+      <x:c r="E95" s="47" t="str">
+        <x:v>Tập trung các mã màu chủ đạo cho UI.</x:v>
+      </x:c>
+      <x:c r="F95" s="47" t="str">
+        <x:v>themes.xml, drawable/bg_*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A96" s="50" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B96" s="47" t="str">
+        <x:v>Resource/Value</x:v>
+      </x:c>
+      <x:c r="C96" s="47" t="str">
+        <x:v>app/src/main/res/values/strings.xml</x:v>
+      </x:c>
+      <x:c r="D96" s="47" t="str">
+        <x:v>Kho chuỗi văn bản tổng quát của Android.</x:v>
+      </x:c>
+      <x:c r="E96" s="47" t="str">
+        <x:v>Nơi nên đặt string dùng lại nếu cần chuẩn hóa thêm.</x:v>
+      </x:c>
+      <x:c r="F96" s="47" t="str">
+        <x:v>layout/*.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="134.27734375" hidden="0" customHeight="1">
+      <x:c r="A97" s="50" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B97" s="47" t="str">
+        <x:v>Resource/Theme</x:v>
+      </x:c>
+      <x:c r="C97" s="47" t="str">
+        <x:v>app/src/main/res/values/themes.xml</x:v>
+      </x:c>
+      <x:c r="D97" s="47" t="str">
+        <x:v>Theme sáng và mặc định của ứng dụng.</x:v>
+      </x:c>
+      <x:c r="E97" s="47" t="str">
+        <x:v>Quy định màu chủ đạo, status bar, navigation bar và window background.</x:v>
+      </x:c>
+      <x:c r="F97" s="47" t="str">
+        <x:v>themes-night/themes.xml, MainActivity.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A98" s="50" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B98" s="47" t="str">
+        <x:v>Resource/XML</x:v>
+      </x:c>
+      <x:c r="C98" s="47" t="str">
+        <x:v>app/src/main/res/xml/backup_rules.xml</x:v>
+      </x:c>
+      <x:c r="D98" s="47" t="str">
+        <x:v>Cấu hình auto backup Android.</x:v>
+      </x:c>
+      <x:c r="E98" s="47" t="str">
+        <x:v>Điều khiển phạm vi dữ liệu được backup/restore.</x:v>
+      </x:c>
+      <x:c r="F98" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A99" s="50" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B99" s="47" t="str">
+        <x:v>Resource/XML</x:v>
+      </x:c>
+      <x:c r="C99" s="47" t="str">
+        <x:v>app/src/main/res/xml/data_extraction_rules.xml</x:v>
+      </x:c>
+      <x:c r="D99" s="47" t="str">
+        <x:v>Cấu hình data extraction cho Android 12+.</x:v>
+      </x:c>
+      <x:c r="E99" s="47" t="str">
+        <x:v>Kiểm soát dữ liệu cho backup và transfer.</x:v>
+      </x:c>
+      <x:c r="F99" s="47" t="str">
+        <x:v>AndroidManifest.xml</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="107.421875" hidden="0" customHeight="1">
+      <x:c r="A100" s="50" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B100" s="47" t="str">
+        <x:v>Cấu hình gốc</x:v>
+      </x:c>
+      <x:c r="C100" s="47" t="str">
+        <x:v>build.gradle.kts</x:v>
+      </x:c>
+      <x:c r="D100" s="47" t="str">
+        <x:v>Khai báo pluginManagement và repository dùng cho toàn project.</x:v>
+      </x:c>
+      <x:c r="E100" s="47" t="str">
+        <x:v>Điểm khởi tạo Gradle ở cấp root.</x:v>
+      </x:c>
+      <x:c r="F100" s="47" t="str">
+        <x:v>settings.gradle.kts, app/build.gradle.kts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="147.705078125" hidden="0" customHeight="1">
+      <x:c r="A101" s="50" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B101" s="47" t="str">
+        <x:v>Tài liệu</x:v>
+      </x:c>
+      <x:c r="C101" s="47" t="str">
+        <x:v>FIREBASE_MAPS_SETUP.md</x:v>
+      </x:c>
+      <x:c r="D101" s="47" t="str">
+        <x:v>Tài liệu hướng dẫn cấu hình Firebase Storage, Google Maps, SHA1 và kiểm tra nhanh.</x:v>
+      </x:c>
+      <x:c r="E101" s="47" t="str">
+        <x:v>Giúp đồng bộ console Firebase/Google Cloud với mã nguồn hiện tại.</x:v>
+      </x:c>
+      <x:c r="F101" s="47" t="str">
+        <x:v>app/src/google-services.json, AndroidManifest.xml, firestore.rules, storage.rules</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="147.705078125" hidden="0" customHeight="1">
+      <x:c r="A102" s="50" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B102" s="47" t="str">
         <x:v>Bảo mật Firebase</x:v>
       </x:c>
-      <x:c r="C83" s="47" t="str">
+      <x:c r="C102" s="47" t="str">
+        <x:v>firestore.rules</x:v>
+      </x:c>
+      <x:c r="D102" s="47" t="str">
+        <x:v>Luật truy cập Firestore cho users, posts, conversations, messages và notifications.</x:v>
+      </x:c>
+      <x:c r="E102" s="47" t="str">
+        <x:v>Bảo vệ dữ liệu chat, bài đăng và hồ sơ trên Firestore.</x:v>
+      </x:c>
+      <x:c r="F102" s="47" t="str">
+        <x:v>storage.rules, app/src/google-services.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A103" s="50" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B103" s="47" t="str">
+        <x:v>Cấu hình gốc</x:v>
+      </x:c>
+      <x:c r="C103" s="47" t="str">
+        <x:v>gradle.properties</x:v>
+      </x:c>
+      <x:c r="D103" s="47" t="str">
+        <x:v>Thiết lập JVM args, AndroidX và tối ưu build.</x:v>
+      </x:c>
+      <x:c r="E103" s="47" t="str">
+        <x:v>Điều chỉnh hành vi Gradle trên máy phát triển.</x:v>
+      </x:c>
+      <x:c r="F103" s="47" t="str">
+        <x:v>build.gradle.kts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A104" s="50" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B104" s="47" t="str">
+        <x:v>Công cụ build</x:v>
+      </x:c>
+      <x:c r="C104" s="47" t="str">
+        <x:v>gradlew</x:v>
+      </x:c>
+      <x:c r="D104" s="47" t="str">
+        <x:v>Wrapper script cho Gradle trên Unix/Linux/macOS.</x:v>
+      </x:c>
+      <x:c r="E104" s="47" t="str">
+        <x:v>Cho phép build mà không cần cài Gradle toàn cục.</x:v>
+      </x:c>
+      <x:c r="F104" s="47" t="str">
+        <x:v>gradlew.bat, gradle/wrapper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="80.56640625" hidden="0" customHeight="1">
+      <x:c r="A105" s="50" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B105" s="47" t="str">
+        <x:v>Công cụ build</x:v>
+      </x:c>
+      <x:c r="C105" s="47" t="str">
+        <x:v>gradlew.bat</x:v>
+      </x:c>
+      <x:c r="D105" s="47" t="str">
+        <x:v>Wrapper script cho Gradle trên Windows.</x:v>
+      </x:c>
+      <x:c r="E105" s="47" t="str">
+        <x:v>Lệnh chuẩn để build dự án trên máy Windows.</x:v>
+      </x:c>
+      <x:c r="F105" s="47" t="str">
+        <x:v>gradlew, gradle/wrapper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A106" s="50" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B106" s="47" t="str">
+        <x:v>Cấu hình gốc</x:v>
+      </x:c>
+      <x:c r="C106" s="47" t="str">
+        <x:v>settings.gradle.kts</x:v>
+      </x:c>
+      <x:c r="D106" s="47" t="str">
+        <x:v>Đặt tên project BTLAND và include module app.</x:v>
+      </x:c>
+      <x:c r="E106" s="47" t="str">
+        <x:v>Xác định cấu trúc module mà Gradle sẽ build.</x:v>
+      </x:c>
+      <x:c r="F106" s="47" t="str">
+        <x:v>build.gradle.kts, app/build.gradle.kts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="93.994140625" hidden="0" customHeight="1">
+      <x:c r="A107" s="50" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B107" s="47" t="str">
+        <x:v>Bảo mật Firebase</x:v>
+      </x:c>
+      <x:c r="C107" s="47" t="str">
         <x:v>storage.rules</x:v>
       </x:c>
-      <x:c r="D83" s="47" t="str">
+      <x:c r="D107" s="47" t="str">
         <x:v>Luật truy cập Firebase Storage cho ảnh bài đăng và avatar.</x:v>
       </x:c>
-      <x:c r="E83" s="47" t="str">
+      <x:c r="E107" s="47" t="str">
         <x:v>Kiểm soát quyền đọc/ghi ảnh trên Storage.</x:v>
       </x:c>
-      <x:c r="F83" s="47" t="str">
+      <x:c r="F107" s="47" t="str">
         <x:v>firestore.rules, app/src/google-services.json</x:v>
       </x:c>
     </x:row>

</xml_diff>